<commit_message>
chore: refresh HIRA material outputs
</commit_message>
<xml_diff>
--- a/hira_material_automation/output/master/040019__nonmetal_anchor__master.xlsx
+++ b/hira_material_automation/output/master/040019__nonmetal_anchor__master.xlsx
@@ -11,7 +11,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="meta" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'data'!$A$1:$J$2</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'data'!$A$1:$J$3</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -426,7 +426,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J2"/>
+  <dimension ref="A1:J3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -496,43 +496,81 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
+          <t>2020년 01월</t>
+        </is>
+      </c>
+      <c r="B2" t="n">
+        <v>2020</v>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>040019</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>비금속성 ANCHOR</t>
+        </is>
+      </c>
+      <c r="E2" t="n">
+        <v>20573</v>
+      </c>
+      <c r="F2" t="n">
+        <v>4285939178</v>
+      </c>
+      <c r="G2" t="n">
+        <v>695</v>
+      </c>
+      <c r="H2" t="n">
+        <v>142550377</v>
+      </c>
+      <c r="I2" t="n">
+        <v>21268</v>
+      </c>
+      <c r="J2" t="n">
+        <v>4428489555</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
           <t>2026년 01월</t>
         </is>
       </c>
-      <c r="B2" t="n">
+      <c r="B3" t="n">
         <v>2026</v>
       </c>
-      <c r="C2" t="inlineStr">
+      <c r="C3" t="inlineStr">
         <is>
           <t>040019</t>
         </is>
       </c>
-      <c r="D2" t="inlineStr">
+      <c r="D3" t="inlineStr">
         <is>
           <t>비금속성 ANCHOR</t>
         </is>
       </c>
-      <c r="E2" t="n">
+      <c r="E3" t="n">
         <v>25458</v>
       </c>
-      <c r="F2" t="n">
+      <c r="F3" t="n">
         <v>5640311240</v>
       </c>
-      <c r="G2" t="n">
+      <c r="G3" t="n">
         <v>1021</v>
       </c>
-      <c r="H2" t="n">
+      <c r="H3" t="n">
         <v>224685140</v>
       </c>
-      <c r="I2" t="n">
+      <c r="I3" t="n">
         <v>26479</v>
       </c>
-      <c r="J2" t="n">
+      <c r="J3" t="n">
         <v>5864996380</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:J2"/>
+  <autoFilter ref="A1:J3"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -570,7 +608,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2026-03-15T23:13:44+09:00</t>
+          <t>2026-03-16T14:58:29+09:00</t>
         </is>
       </c>
     </row>
@@ -605,237 +643,10 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
-</file>
-
-<file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="문서" ma:contentTypeID="0x0101003A7F18B03E33BF4DA150962F23733248" ma:contentTypeVersion="13" ma:contentTypeDescription="새 문서를 만듭니다." ma:contentTypeScope="" ma:versionID="00d5bc73201a7cf16b7b67444666f865">
-  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="9bf3fbf4-c6f4-4df2-8cf6-49e28bf51f66" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="aa075d809ae3b8704ec3701444232834" ns2:_="">
-    <xsd:import namespace="9bf3fbf4-c6f4-4df2-8cf6-49e28bf51f66"/>
-    <xsd:element name="properties">
-      <xsd:complexType>
-        <xsd:sequence>
-          <xsd:element name="documentManagement">
-            <xsd:complexType>
-              <xsd:all>
-                <xsd:element ref="ns2:MediaServiceMetadata" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceFastMetadata" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceSearchProperties" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceObjectDetectorVersions" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceDateTaken" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceGenerationTime" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceEventHashCode" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaLengthInSeconds" minOccurs="0"/>
-                <xsd:element ref="ns2:lcf76f155ced4ddcb4097134ff3c332f" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceOCR" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceLocation" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceBillingMetadata" minOccurs="0"/>
-              </xsd:all>
-            </xsd:complexType>
-          </xsd:element>
-        </xsd:sequence>
-      </xsd:complexType>
-    </xsd:element>
-  </xsd:schema>
-  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:dms="http://schemas.microsoft.com/office/2006/documentManagement/types" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" targetNamespace="9bf3fbf4-c6f4-4df2-8cf6-49e28bf51f66" elementFormDefault="qualified">
-    <xsd:import namespace="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <xsd:import namespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <xsd:element name="MediaServiceMetadata" ma:index="8" nillable="true" ma:displayName="MediaServiceMetadata" ma:hidden="true" ma:internalName="MediaServiceMetadata" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Note"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaServiceFastMetadata" ma:index="9" nillable="true" ma:displayName="MediaServiceFastMetadata" ma:hidden="true" ma:internalName="MediaServiceFastMetadata" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Note"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaServiceSearchProperties" ma:index="10" nillable="true" ma:displayName="MediaServiceSearchProperties" ma:hidden="true" ma:internalName="MediaServiceSearchProperties" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Note"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaServiceObjectDetectorVersions" ma:index="11" nillable="true" ma:displayName="MediaServiceObjectDetectorVersions" ma:hidden="true" ma:indexed="true" ma:internalName="MediaServiceObjectDetectorVersions" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Text"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaServiceDateTaken" ma:index="12" nillable="true" ma:displayName="MediaServiceDateTaken" ma:hidden="true" ma:indexed="true" ma:internalName="MediaServiceDateTaken" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Text"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaServiceGenerationTime" ma:index="13" nillable="true" ma:displayName="MediaServiceGenerationTime" ma:hidden="true" ma:internalName="MediaServiceGenerationTime" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Text"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaServiceEventHashCode" ma:index="14" nillable="true" ma:displayName="MediaServiceEventHashCode" ma:hidden="true" ma:internalName="MediaServiceEventHashCode" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Text"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaLengthInSeconds" ma:index="15" nillable="true" ma:displayName="MediaLengthInSeconds" ma:hidden="true" ma:internalName="MediaLengthInSeconds" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Unknown"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="lcf76f155ced4ddcb4097134ff3c332f" ma:index="17" nillable="true" ma:taxonomy="true" ma:internalName="lcf76f155ced4ddcb4097134ff3c332f" ma:taxonomyFieldName="MediaServiceImageTags" ma:displayName="이미지 태그" ma:readOnly="false" ma:fieldId="{5cf76f15-5ced-4ddc-b409-7134ff3c332f}" ma:taxonomyMulti="true" ma:sspId="450bca00-d6b9-4d94-bef9-41f99f1b5cd1" ma:termSetId="09814cd3-568e-fe90-9814-8d621ff8fb84" ma:anchorId="fba54fb3-c3e1-fe81-a776-ca4b69148c4d" ma:open="true" ma:isKeyword="false">
-      <xsd:complexType>
-        <xsd:sequence>
-          <xsd:element ref="pc:Terms" minOccurs="0" maxOccurs="1"/>
-        </xsd:sequence>
-      </xsd:complexType>
-    </xsd:element>
-    <xsd:element name="MediaServiceOCR" ma:index="18" nillable="true" ma:displayName="Extracted Text" ma:internalName="MediaServiceOCR" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Note">
-          <xsd:maxLength value="255"/>
-        </xsd:restriction>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaServiceLocation" ma:index="19" nillable="true" ma:displayName="Location" ma:indexed="true" ma:internalName="MediaServiceLocation" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Text"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaServiceBillingMetadata" ma:index="20" nillable="true" ma:displayName="MediaServiceBillingMetadata" ma:hidden="true" ma:internalName="MediaServiceBillingMetadata" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Note"/>
-      </xsd:simpleType>
-    </xsd:element>
-  </xsd:schema>
-  <xsd:schema xmlns="http://schemas.openxmlformats.org/package/2006/metadata/core-properties" xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:dc="http://purl.org/dc/elements/1.1/" xmlns:dcterms="http://purl.org/dc/terms/" xmlns:odoc="http://schemas.microsoft.com/internal/obd" targetNamespace="http://schemas.openxmlformats.org/package/2006/metadata/core-properties" elementFormDefault="qualified" attributeFormDefault="unqualified" blockDefault="#all">
-    <xsd:import namespace="http://purl.org/dc/elements/1.1/" schemaLocation="http://dublincore.org/schemas/xmls/qdc/2003/04/02/dc.xsd"/>
-    <xsd:import namespace="http://purl.org/dc/terms/" schemaLocation="http://dublincore.org/schemas/xmls/qdc/2003/04/02/dcterms.xsd"/>
-    <xsd:element name="coreProperties" type="CT_coreProperties"/>
-    <xsd:complexType name="CT_coreProperties">
-      <xsd:all>
-        <xsd:element ref="dc:creator" minOccurs="0" maxOccurs="1"/>
-        <xsd:element ref="dcterms:created" minOccurs="0" maxOccurs="1"/>
-        <xsd:element ref="dc:identifier" minOccurs="0" maxOccurs="1"/>
-        <xsd:element name="contentType" minOccurs="0" maxOccurs="1" type="xsd:string" ma:index="0" ma:displayName="콘텐츠 형식"/>
-        <xsd:element ref="dc:title" minOccurs="0" maxOccurs="1" ma:index="4" ma:displayName="제목"/>
-        <xsd:element ref="dc:subject" minOccurs="0" maxOccurs="1"/>
-        <xsd:element ref="dc:description" minOccurs="0" maxOccurs="1"/>
-        <xsd:element name="keywords" minOccurs="0" maxOccurs="1" type="xsd:string"/>
-        <xsd:element ref="dc:language" minOccurs="0" maxOccurs="1"/>
-        <xsd:element name="category" minOccurs="0" maxOccurs="1" type="xsd:string"/>
-        <xsd:element name="version" minOccurs="0" maxOccurs="1" type="xsd:string"/>
-        <xsd:element name="revision" minOccurs="0" maxOccurs="1" type="xsd:string">
-          <xsd:annotation>
-            <xsd:documentation>
-                        This value indicates the number of saves or revisions. The application is responsible for updating this value after each revision.
-                    </xsd:documentation>
-          </xsd:annotation>
-        </xsd:element>
-        <xsd:element name="lastModifiedBy" minOccurs="0" maxOccurs="1" type="xsd:string"/>
-        <xsd:element ref="dcterms:modified" minOccurs="0" maxOccurs="1"/>
-        <xsd:element name="contentStatus" minOccurs="0" maxOccurs="1" type="xsd:string"/>
-      </xsd:all>
-    </xsd:complexType>
-  </xsd:schema>
-  <xs:schema xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" xmlns:xs="http://www.w3.org/2001/XMLSchema" targetNamespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" elementFormDefault="qualified" attributeFormDefault="unqualified">
-    <xs:element name="Person">
-      <xs:complexType>
-        <xs:sequence>
-          <xs:element ref="pc:DisplayName" minOccurs="0"/>
-          <xs:element ref="pc:AccountId" minOccurs="0"/>
-          <xs:element ref="pc:AccountType" minOccurs="0"/>
-        </xs:sequence>
-      </xs:complexType>
-    </xs:element>
-    <xs:element name="DisplayName" type="xs:string"/>
-    <xs:element name="AccountId" type="xs:string"/>
-    <xs:element name="AccountType" type="xs:string"/>
-    <xs:element name="BDCAssociatedEntity">
-      <xs:complexType>
-        <xs:sequence>
-          <xs:element ref="pc:BDCEntity" minOccurs="0" maxOccurs="unbounded"/>
-        </xs:sequence>
-        <xs:attribute ref="pc:EntityNamespace"/>
-        <xs:attribute ref="pc:EntityName"/>
-        <xs:attribute ref="pc:SystemInstanceName"/>
-        <xs:attribute ref="pc:AssociationName"/>
-      </xs:complexType>
-    </xs:element>
-    <xs:attribute name="EntityNamespace" type="xs:string"/>
-    <xs:attribute name="EntityName" type="xs:string"/>
-    <xs:attribute name="SystemInstanceName" type="xs:string"/>
-    <xs:attribute name="AssociationName" type="xs:string"/>
-    <xs:element name="BDCEntity">
-      <xs:complexType>
-        <xs:sequence>
-          <xs:element ref="pc:EntityDisplayName" minOccurs="0"/>
-          <xs:element ref="pc:EntityInstanceReference" minOccurs="0"/>
-          <xs:element ref="pc:EntityId1" minOccurs="0"/>
-          <xs:element ref="pc:EntityId2" minOccurs="0"/>
-          <xs:element ref="pc:EntityId3" minOccurs="0"/>
-          <xs:element ref="pc:EntityId4" minOccurs="0"/>
-          <xs:element ref="pc:EntityId5" minOccurs="0"/>
-        </xs:sequence>
-      </xs:complexType>
-    </xs:element>
-    <xs:element name="EntityDisplayName" type="xs:string"/>
-    <xs:element name="EntityInstanceReference" type="xs:string"/>
-    <xs:element name="EntityId1" type="xs:string"/>
-    <xs:element name="EntityId2" type="xs:string"/>
-    <xs:element name="EntityId3" type="xs:string"/>
-    <xs:element name="EntityId4" type="xs:string"/>
-    <xs:element name="EntityId5" type="xs:string"/>
-    <xs:element name="Terms">
-      <xs:complexType>
-        <xs:sequence>
-          <xs:element ref="pc:TermInfo" minOccurs="0" maxOccurs="unbounded"/>
-        </xs:sequence>
-      </xs:complexType>
-    </xs:element>
-    <xs:element name="TermInfo">
-      <xs:complexType>
-        <xs:sequence>
-          <xs:element ref="pc:TermName" minOccurs="0"/>
-          <xs:element ref="pc:TermId" minOccurs="0"/>
-        </xs:sequence>
-      </xs:complexType>
-    </xs:element>
-    <xs:element name="TermName" type="xs:string"/>
-    <xs:element name="TermId" type="xs:string"/>
-  </xs:schema>
-</ct:contentTypeSchema>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="9bf3fbf4-c6f4-4df2-8cf6-49e28bf51f66">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-  </documentManagement>
-</p:properties>
-</file>
-
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{BB3C3B49-8AA3-456B-A8D3-F66384232155}"/>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{97E420CD-CC1F-4301-A9E9-64A670FEDA55}"/>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{AF05E770-0B4E-4FAE-A800-4AEEDC23C857}"/>
 </file>
</xml_diff>